<commit_message>
feat: enforce uppercase inputs, mandate banking details, update Cadastro E-mail sheet columns and add migration
</commit_message>
<xml_diff>
--- a/supabase/Borderô para cadastro E-mail.xlsx
+++ b/supabase/Borderô para cadastro E-mail.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="21727"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FFC48212-281F-4DDC-9D21-1BBE4558899B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CA891D7-66F2-4193-B2CD-994E9FC51BA1}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Detalhado" sheetId="1" r:id="rId1"/>
@@ -13,11 +13,18 @@
     <sheet name="Cadastro E-mail" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="77">
   <si>
     <t>Borderô 30/05/2026 - Lote 2</t>
   </si>
@@ -217,9 +224,6 @@
     <t>Carteira</t>
   </si>
   <si>
-    <t>Empresa</t>
-  </si>
-  <si>
     <t>Somente últimos numeros do campo empresa ativação</t>
   </si>
   <si>
@@ -236,6 +240,21 @@
   </si>
   <si>
     <t>Em branco</t>
+  </si>
+  <si>
+    <t>Restam</t>
+  </si>
+  <si>
+    <t>Total de Parcelas tela vendas</t>
+  </si>
+  <si>
+    <t>Selecionadas tela vendas</t>
+  </si>
+  <si>
+    <t>Deve ser nesse formato Mês / Ano</t>
+  </si>
+  <si>
+    <t>Campo Empresa da tela de vendas</t>
   </si>
 </sst>
 </file>
@@ -300,7 +319,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -310,6 +329,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -365,7 +390,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -383,11 +408,8 @@
     <xf numFmtId="4" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -397,16 +419,25 @@
     <xf numFmtId="14" fontId="6" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="17" fontId="5" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="17" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -748,7 +779,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:S6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
@@ -771,30 +802,30 @@
     <col min="19" max="19" width="19" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:19" ht="31.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
-      <c r="H1" s="7"/>
-      <c r="I1" s="7"/>
-      <c r="J1" s="7"/>
-      <c r="K1" s="7"/>
-      <c r="L1" s="7"/>
-      <c r="M1" s="7"/>
-      <c r="N1" s="7"/>
-      <c r="O1" s="7"/>
-      <c r="P1" s="7"/>
-      <c r="Q1" s="7"/>
-      <c r="R1" s="7"/>
-      <c r="S1" s="7"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
+      <c r="L1" s="17"/>
+      <c r="M1" s="17"/>
+      <c r="N1" s="17"/>
+      <c r="O1" s="17"/>
+      <c r="P1" s="17"/>
+      <c r="Q1" s="17"/>
+      <c r="R1" s="17"/>
+      <c r="S1" s="17"/>
     </row>
-    <row r="2" spans="1:19" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:19" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -853,7 +884,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:19" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:19" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>19</v>
       </c>
@@ -912,7 +943,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="4" spans="1:19" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:19" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>33</v>
       </c>
@@ -971,7 +1002,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="5" spans="1:19" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:19" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>36</v>
       </c>
@@ -1030,7 +1061,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="6" spans="1:19" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:19" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
@@ -1058,7 +1089,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:P5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
     <col min="2" max="2" width="8" customWidth="1"/>
@@ -1078,27 +1109,27 @@
     <col min="16" max="16" width="21" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:16" ht="31.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
-      <c r="H1" s="7"/>
-      <c r="I1" s="7"/>
-      <c r="J1" s="7"/>
-      <c r="K1" s="7"/>
-      <c r="L1" s="7"/>
-      <c r="M1" s="7"/>
-      <c r="N1" s="7"/>
-      <c r="O1" s="7"/>
-      <c r="P1" s="7"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
+      <c r="L1" s="17"/>
+      <c r="M1" s="17"/>
+      <c r="N1" s="17"/>
+      <c r="O1" s="17"/>
+      <c r="P1" s="17"/>
     </row>
-    <row r="2" spans="1:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -1148,7 +1179,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>20</v>
       </c>
@@ -1198,7 +1229,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="4" spans="1:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -1248,7 +1279,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5"/>
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
@@ -1274,250 +1305,264 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9CEBD5A4-557F-4019-99B5-BF42B12D36C0}">
-  <dimension ref="A1:AG3"/>
-  <sheetFormatPr defaultColWidth="6.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:AH3"/>
+  <sheetFormatPr defaultColWidth="6.33203125" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.7109375" style="9" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.140625" style="9" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.28515625" style="9" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.85546875" style="9" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.7109375" style="9" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.5703125" style="9" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14" style="9" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.85546875" style="9" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="7.42578125" style="9" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="5.140625" style="9" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="6.7109375" style="9" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="5.140625" style="9" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.7109375" style="9" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="5.140625" style="9" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="9.85546875" style="9" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="8" style="9" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="6.28515625" style="9"/>
-    <col min="18" max="18" width="8" style="9" bestFit="1" customWidth="1"/>
-    <col min="19" max="20" width="3.5703125" style="9" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10" style="9" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="3.5703125" style="9" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="11.7109375" style="9" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11" style="9" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="5.85546875" style="9" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="7.42578125" style="9" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="11.28515625" style="9" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="15.140625" style="9" bestFit="1" customWidth="1"/>
-    <col min="29" max="16384" width="6.28515625" style="9"/>
+    <col min="1" max="1" width="16.6640625" style="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.109375" style="8" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.33203125" style="8" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.88671875" style="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.6640625" style="8" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.5546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14" style="8" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.88671875" style="8" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.44140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="5.109375" style="8" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="19.44140625" style="8" customWidth="1"/>
+    <col min="12" max="12" width="5.109375" style="8" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12" style="8" customWidth="1"/>
+    <col min="14" max="14" width="8.6640625" style="8" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="5.109375" style="8" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="9.88671875" style="8" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="8" style="8" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="6.33203125" style="8"/>
+    <col min="19" max="19" width="8" style="8" bestFit="1" customWidth="1"/>
+    <col min="20" max="21" width="3.5546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="10" style="8" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="3.5546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.6640625" style="8" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="11" style="8" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="5.88671875" style="8" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="7.44140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="11.33203125" style="8" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="15.109375" style="8" bestFit="1" customWidth="1"/>
+    <col min="30" max="16384" width="6.33203125" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A1" s="10" t="s">
+    <row r="1" spans="1:34" x14ac:dyDescent="0.3">
+      <c r="A1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="F1" s="10" t="s">
+      <c r="F1" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="G1" s="10" t="s">
+      <c r="G1" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="H1" s="10" t="s">
+      <c r="H1" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="I1" s="10" t="s">
+      <c r="I1" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="J1" s="10" t="s">
+      <c r="J1" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="K1" s="10" t="s">
+      <c r="K1" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="L1" s="10" t="s">
+      <c r="L1" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="M1" s="10" t="s">
+      <c r="M1" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="N1" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="N1" s="10" t="s">
+      <c r="O1" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="O1" s="10" t="s">
+      <c r="P1" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="P1" s="10" t="s">
+      <c r="Q1" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="Q1" s="10" t="s">
+      <c r="R1" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="R1" s="10" t="s">
+      <c r="S1" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="S1" s="10" t="s">
+      <c r="T1" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="T1" s="10" t="s">
+      <c r="U1" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="U1" s="10" t="s">
+      <c r="V1" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="V1" s="10" t="s">
+      <c r="W1" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="W1" s="10" t="s">
+      <c r="X1" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="X1" s="10" t="s">
+      <c r="Y1" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="Y1" s="11" t="s">
+      <c r="Z1" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="Z1" s="11" t="s">
+      <c r="AA1" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="AA1" s="11" t="s">
+      <c r="AB1" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="AB1" s="11" t="s">
+      <c r="AC1" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="AC1" s="8"/>
-      <c r="AD1" s="8"/>
-      <c r="AE1" s="8"/>
-      <c r="AF1" s="8"/>
-      <c r="AG1" s="8"/>
+      <c r="AD1" s="7"/>
+      <c r="AE1" s="7"/>
+      <c r="AF1" s="7"/>
+      <c r="AG1" s="7"/>
+      <c r="AH1" s="7"/>
     </row>
-    <row r="2" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A2" s="11" t="s">
+    <row r="2" spans="1:34" x14ac:dyDescent="0.3">
+      <c r="A2" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="B2" s="11">
+      <c r="B2" s="10">
         <v>10459</v>
       </c>
-      <c r="C2" s="11">
+      <c r="C2" s="10">
         <v>26</v>
       </c>
-      <c r="D2" s="11">
+      <c r="D2" s="10">
         <v>11878</v>
       </c>
-      <c r="E2" s="12">
+      <c r="E2" s="11">
         <v>46172</v>
       </c>
-      <c r="F2" s="13" t="s">
+      <c r="F2" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="G2" s="11" t="s">
+      <c r="G2" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="H2" s="11" t="s">
+      <c r="H2" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="I2" s="11">
+      <c r="I2" s="10">
         <v>21</v>
       </c>
-      <c r="J2" s="14"/>
-      <c r="K2" s="15">
+      <c r="J2" s="13"/>
+      <c r="K2" s="14">
         <v>46174</v>
       </c>
-      <c r="L2" s="14"/>
-      <c r="M2" s="11">
+      <c r="L2" s="13"/>
+      <c r="M2" s="13"/>
+      <c r="N2" s="10">
         <v>1</v>
       </c>
-      <c r="N2" s="14"/>
-      <c r="O2" s="14"/>
-      <c r="P2" s="11" t="s">
+      <c r="O2" s="13"/>
+      <c r="P2" s="13"/>
+      <c r="Q2" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="Q2" s="11">
+      <c r="R2" s="10">
         <v>104</v>
       </c>
-      <c r="R2" s="11">
+      <c r="S2" s="10">
         <v>4056</v>
       </c>
-      <c r="S2" s="14"/>
-      <c r="T2" s="14"/>
-      <c r="U2" s="11">
+      <c r="T2" s="13"/>
+      <c r="U2" s="13"/>
+      <c r="V2" s="10">
         <v>589284685</v>
       </c>
-      <c r="V2" s="11">
+      <c r="W2" s="10">
         <v>3</v>
       </c>
-      <c r="W2" s="11">
+      <c r="X2" s="10">
         <v>300</v>
       </c>
-      <c r="X2" s="11">
+      <c r="Y2" s="10">
         <v>186.6</v>
       </c>
-      <c r="Y2" s="11" t="s">
+      <c r="Z2" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="Z2" s="11">
+      <c r="AA2" s="10">
         <v>113.4</v>
       </c>
-      <c r="AA2" s="11">
+      <c r="AB2" s="10">
         <v>0.378</v>
       </c>
-      <c r="AB2" s="11">
+      <c r="AC2" s="10">
         <v>71942</v>
       </c>
     </row>
-    <row r="3" spans="1:33" s="16" customFormat="1" ht="73.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="16" t="s">
+    <row r="3" spans="1:34" s="15" customFormat="1" ht="73.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="15" t="s">
+        <v>66</v>
+      </c>
+      <c r="H3" s="16" t="s">
+        <v>76</v>
+      </c>
+      <c r="J3" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="K3" s="19" t="s">
+        <v>75</v>
+      </c>
+      <c r="L3" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="M3" s="16" t="s">
+        <v>73</v>
+      </c>
+      <c r="N3" s="16" t="s">
+        <v>74</v>
+      </c>
+      <c r="O3" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q3" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="R3" s="18" t="s">
         <v>67</v>
       </c>
-      <c r="H3" s="16" t="s">
-        <v>66</v>
-      </c>
-      <c r="J3" s="16" t="s">
-        <v>72</v>
-      </c>
-      <c r="L3" s="16" t="s">
-        <v>72</v>
-      </c>
-      <c r="N3" s="16" t="s">
-        <v>72</v>
-      </c>
-      <c r="P3" s="16" t="s">
-        <v>65</v>
-      </c>
-      <c r="Q3" s="17" t="s">
+      <c r="S3" s="18"/>
+      <c r="T3" s="18"/>
+      <c r="U3" s="18"/>
+      <c r="V3" s="18"/>
+      <c r="W3" s="18"/>
+      <c r="X3" s="15" t="s">
         <v>68</v>
       </c>
-      <c r="R3" s="17"/>
-      <c r="S3" s="17"/>
-      <c r="T3" s="17"/>
-      <c r="U3" s="17"/>
-      <c r="V3" s="17"/>
-      <c r="W3" s="16" t="s">
+      <c r="Y3" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="X3" s="16" t="s">
+      <c r="AA3" s="15" t="s">
         <v>70</v>
       </c>
-      <c r="Z3" s="16" t="s">
+      <c r="AB3" s="15" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC3" s="15" t="s">
         <v>71</v>
-      </c>
-      <c r="AA3" s="16" t="s">
-        <v>58</v>
-      </c>
-      <c r="AB3" s="16" t="s">
-        <v>72</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="Q3:V3"/>
+    <mergeCell ref="R3:W3"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>